<commit_message>
this is first commit
</commit_message>
<xml_diff>
--- a/ITVEDANTCLASS1.xlsx
+++ b/ITVEDANTCLASS1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sayyed\Downloads\Dmart_Sales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{478EDE62-910B-4FD9-AFB9-5D41B479357E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E495B825-4D88-47D5-9F1D-CBE09FC20707}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{2A9389EE-B0A1-435E-B258-E712E71DF2EE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{2A9389EE-B0A1-435E-B258-E712E71DF2EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1738,7 +1738,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2171A7E-7404-4D83-A0CF-0854A0E0AA58}">
-  <dimension ref="A2:E6"/>
+  <dimension ref="A2:E15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -1851,6 +1851,36 @@
         <v>21</v>
       </c>
     </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C11">
+        <f>SUM('2023:2025'!B3)</f>
+        <v>212</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C12">
+        <f>SUM('2023:2025'!B4)</f>
+        <v>280</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C13">
+        <f>SUM('2023:2025'!B5)</f>
+        <v>232</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C14">
+        <f>SUM('2023:2025'!B6)</f>
+        <v>112</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C15">
+        <f>SUM('2023:2025'!B7)</f>
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>